<commit_message>
Fixed column 1 label name
</commit_message>
<xml_diff>
--- a/Data/Table1_clean.xlsx
+++ b/Data/Table1_clean.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/connorpiercy/Documents/GitHub/Group_8_Project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/connorpiercy/Documents/GitHub/Group_8_Project/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{388D2757-ABDC-AD4C-B3B9-0F592660640B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37F70BD5-6EE5-B049-BCE3-A8E1ECBCA2D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="13980" yWindow="600" windowWidth="14820" windowHeight="16660" xr2:uid="{D913AFE5-FFEF-D343-BAB9-A12C62385E55}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="56">
   <si>
     <t>11-Na*</t>
   </si>
@@ -204,6 +204,9 @@
   </si>
   <si>
     <t>[0.00]</t>
+  </si>
+  <si>
+    <t>Elements</t>
   </si>
 </sst>
 </file>
@@ -589,6 +592,9 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>55</v>
+      </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>

</xml_diff>